<commit_message>
working on duplicate proposals
</commit_message>
<xml_diff>
--- a/proposal_output/proposals.xlsx
+++ b/proposal_output/proposals.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proposals'!$A$1:$O$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Workplan'!$A$1:$G$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Website Register'!$A$1:$G$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Keywords'!$A$1:$D$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Keywords'!$A$1:$D$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Content Calendar'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Workflow Queue'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Workflows'!$A$1:$E$5</definedName>
@@ -445,14 +445,14 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="43" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
-    <col width="54" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
@@ -540,12 +540,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>bc97777e6c0833cb</t>
+          <t>17b2c29e5c65d88f</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Open University of Kenya Tender Notice.pdf</t>
+          <t>Open University of Kenya Prequalification of Suppliers (2026-2028)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>training</t>
+          <t>training, ICT training</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -578,12 +578,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Matched configured ICT keyword(s): training.</t>
+          <t>The tender prequalification includes dedicated categories for 'Provision of ICT Management Consulting, ICT Systems Audit and Training on ICT Security Solutions' and 'Consultancy on E-Learning and Online Systems'.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Review source document for eligibility requirements.</t>
+          <t>Open to all interested and eligible firms. Certain reserved categories are restricted to AGPO groups (Youth, Women, and PWDs) with a valid AGPO certificate.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -609,19 +609,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>166f9b27c5e956f4</t>
+          <t>28f70fbc788b8104</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Blue Dot Network (BDN) Certification</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Certification</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Certification</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>https://www.bluedot-network.org/certification</t>
@@ -639,7 +639,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>apply for certification</t>
+          <t>certification offer, certification application, apply for certification</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -649,12 +649,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Matched configured ICT keyword(s): apply for certification.</t>
+          <t>Offers an official certification process for global infrastructure projects, which explicitly includes the ICT sector.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Review source document for eligibility requirements.</t>
+          <t>Applies to infrastructure projects across energy, water, transport, and ICT, under various delivery and ownership models.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Data science</t>
+          <t>Digital Health &amp; Climate Tech</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>machine learning</t>
+          <t>machine learning, artificial intelligence, grant application, funding opportunity</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -791,12 +791,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Matched configured ICT keyword(s): machine learning.</t>
+          <t>The platform outlines grant funding programs designed to catalyze research and dataset creation at the intersection of climate change and machine learning.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Review source document for eligibility requirements.</t>
+          <t>Collaborations between academic researchers, non-profits, startups, and governmental organizations globally.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -822,17 +822,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>17124d19bfc6b3cd</t>
+          <t>9686535c456d1a83</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Climate Change AI Innovation Grants</t>
+          <t>Climate Change AI Innovation Grants Program</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Data science</t>
+          <t>Digital Health &amp; Climate Tech</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>analysis, machine learning, artificial intelligence, training</t>
+          <t>machine learning, artificial intelligence, data analysis, data science, grant application, funding opportunity</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -862,12 +862,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Matched configured ICT keyword(s): analysis, machine learning, artificial intelligence, training.</t>
+          <t>The program awards seed grants of up to $150K for projects deploying machine learning, data science, and AI tools to address climate change challenges.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Review source document for eligibility requirements.</t>
+          <t>Academic researchers, non-profits, startups, and governmental organizations seeking to build partnerships and public datasets. No active call is currently open, but proposals are kept on file.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1903,11 +1903,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
@@ -2276,8 +2276,188 @@
       </c>
       <c r="D20" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>digital health Africa grant</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Digital Health &amp; Climate Tech</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>AI healthcare Africa funding</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Digital Health &amp; Climate Tech</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>telemedicine Africa grant</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Digital Health &amp; Climate Tech</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>climate technology Africa funding</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Digital Health &amp; Climate Tech</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>smart cities Africa grant</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Digital Health &amp; Climate Tech</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>youth employment Africa grant</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Youth, Women &amp; Inclusion</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>youth digital skills Africa funding</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Youth, Women &amp; Inclusion</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>women in technology Africa funding</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Youth, Women &amp; Inclusion</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>women in STEM Africa grant</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Youth, Women &amp; Inclusion</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>gender inclusion digital Africa grant</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Youth, Women &amp; Inclusion</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D20"/>
+  <autoFilter ref="A1:D30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2401,12 +2581,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>bc97777e6c0833cb</t>
+          <t>17b2c29e5c65d88f</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Open University of Kenya Tender Notice.pdf</t>
+          <t>Open University of Kenya Prequalification of Suppliers (2026-2028)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2541,12 +2721,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>17124d19bfc6b3cd</t>
+          <t>9686535c456d1a83</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Climate Change AI Innovation Grants</t>
+          <t>Climate Change AI Innovation Grants Program</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2560,7 +2740,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -2611,12 +2791,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>166f9b27c5e956f4</t>
+          <t>28f70fbc788b8104</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Certification</t>
+          <t>Blue Dot Network (BDN) Certification</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">

</xml_diff>

<commit_message>
Fix stale scraping: supervise Render schedulers and stop dropping real tenders
The proposal_scheduler.py and mygov_alert_scheduler.py background loops on
Render had no supervision, and /api/health only checks the Next.js server, so
either loop could die silently while the container kept reporting healthy and
proposal_output/ went stale for days. start-render.sh now watches all three
processes and exits (triggering a restart) if any of them dies.

Separately, collect()/collect_raw() applied the per-source max_links cap
before filtering for keyword/discovery-term relevance. On sites with large
navigation menus (e.g. KRA), real tender links sat past that cap and were
silently dropped every run. Filtering now happens before the cap; KRA alone
went from 0 to 13 candidates, and total raw candidates across sources roughly
doubled on the next run.
</commit_message>
<xml_diff>
--- a/proposal_output/proposals.xlsx
+++ b/proposal_output/proposals.xlsx
@@ -540,12 +540,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7b06c862b59f701e</t>
+          <t>8d40238686713191</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Open University of Kenya Tender Notice</t>
+          <t>Open University of Kenya Supplier Prequalification (2026-2028)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -578,12 +578,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Invites registration and prequalification for several ICT-related categories including e-learning systems consultancy, ICT management consulting, and training on ICT security solutions.</t>
+          <t>Tender notice includes a specific open category (OUK/026/OP/2026-2028) for the provision of ICT Management Consulting, ICT Systems Audit, and Training on ICT Security Solutions.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Open to all interested and eligible firms; must submit completed physical prequalification documents to Konza Technopolis.</t>
+          <t>Open to all eligible firms. Prequalification documents must be downloaded from the website and physically deposited by Thursday, 20th August 2026, 11:30 AM East African Time.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -602,19 +602,19 @@
         </is>
       </c>
       <c r="N2" s="2" t="n">
-        <v>46247</v>
+        <v>46253</v>
       </c>
       <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>9cca09bd6a8caab0</t>
+          <t>166f9b27c5e956f4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Blue Dot Network Certification</t>
+          <t>Certification</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>certification application, apply for certification, certification offer</t>
+          <t>apply for certification</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -649,12 +649,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Provides a certification pathway for major infrastructure projects, explicitly including those in the ICT sector.</t>
+          <t>Matched configured ICT keyword(s): apply for certification.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Open to projects across different life cycle stages (planning to operations) and various delivery models. Must meet robust international standards across 10 elements.</t>
+          <t>Review source document for eligibility requirements.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="N3" s="2" t="n">
-        <v>46247</v>
+        <v>46253</v>
       </c>
       <c r="O3" t="inlineStr"/>
     </row>
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="N4" s="2" t="n">
-        <v>46247</v>
+        <v>46253</v>
       </c>
       <c r="O4" t="inlineStr"/>
     </row>
@@ -781,22 +781,22 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>machine learning, artificial intelligence, grant application, funding opportunity</t>
+          <t>machine learning, artificial intelligence, grant application, funding opportunity, climate technology Africa funding</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>The platform outlines grant funding programs designed to catalyze research and dataset creation at the intersection of climate change and machine learning.</t>
+          <t>Provides grant opportunities at the intersection of climate change and machine learning/AI, which aligns with climate technology funding keywords.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Collaborations between academic researchers, non-profits, startups, and governmental organizations globally.</t>
+          <t>Supports research, deployment, and dataset creation. Eligibility varies per specific call (some past calls were Africa-focused).</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="N5" s="2" t="n">
-        <v>46247</v>
+        <v>46253</v>
       </c>
       <c r="O5" t="inlineStr"/>
     </row>
@@ -852,22 +852,22 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>grant application, funding opportunity, artificial intelligence, machine learning</t>
+          <t>artificial intelligence, machine learning, grant application, funding opportunity</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>A seed grant program focusing on the development of AI/ML tools, datasets, and systems to address climate change mitigation and adaptation.</t>
+          <t>Provides seed funding of up to $150K for projects leveraging artificial intelligence and machine learning to tackle climate change mitigation and adaptation.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Allocates seed grants typically up to $150K for projects of one year in duration. No current active calls, but accepts partnership inquiries.</t>
+          <t>Aims to build partnerships between academic researchers, non-profits, startups, and other companies. Currently has no active/future calls planned.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -886,7 +886,7 @@
         </is>
       </c>
       <c r="N6" s="2" t="n">
-        <v>46247</v>
+        <v>46253</v>
       </c>
       <c r="O6" t="inlineStr"/>
     </row>
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="N7" s="2" t="n">
-        <v>46247</v>
+        <v>46253</v>
       </c>
       <c r="O7" t="inlineStr"/>
     </row>
@@ -1028,7 +1028,7 @@
         </is>
       </c>
       <c r="N8" s="2" t="n">
-        <v>46247</v>
+        <v>46253</v>
       </c>
       <c r="O8" t="inlineStr"/>
     </row>
@@ -1099,7 +1099,7 @@
         </is>
       </c>
       <c r="N9" s="2" t="n">
-        <v>46247</v>
+        <v>46253</v>
       </c>
       <c r="O9" t="inlineStr"/>
     </row>
@@ -1176,10 +1176,10 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46247</v>
+        <v>46253</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>46249</v>
+        <v>46255</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1205,10 +1205,10 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>46247</v>
+        <v>46253</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>46249</v>
+        <v>46255</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1238,10 +1238,10 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>46250</v>
+        <v>46256</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>46252</v>
+        <v>46258</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1271,10 +1271,10 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>46250</v>
+        <v>46256</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>46254</v>
+        <v>46260</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1304,10 +1304,10 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>46252</v>
+        <v>46258</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>46259</v>
+        <v>46265</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1337,10 +1337,10 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>46254</v>
+        <v>46260</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>46261</v>
+        <v>46267</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1370,10 +1370,10 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>46261</v>
+        <v>46267</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2581,12 +2581,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7b06c862b59f701e</t>
+          <t>8d40238686713191</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Open University of Kenya Tender Notice</t>
+          <t>Open University of Kenya Supplier Prequalification (2026-2028)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2600,7 +2600,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>46251</v>
+        <v>46253</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2791,12 +2791,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>9cca09bd6a8caab0</t>
+          <t>166f9b27c5e956f4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Blue Dot Network Certification</t>
+          <t>Certification</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">

</xml_diff>

<commit_message>
Wire immediate myGov alerts into the recurring 6-hour scheduler run
proposal_scheduler.py ran proposal_hybrid_monitor.py with no flags, so the
--mygov-alert path (email for newly discovered myGov Kenya opportunities,
tracked in mygov_seen.json) was dead code in production. Only the separate
Tue/Thu digest (mygov_alert_scheduler.py) ever sent mail, and if that loop
died silently, nothing else would notice. Now every scheduled run also
checks for and emails new myGov items, verified locally: this run found and
emailed one new item (8d40238686713191).
</commit_message>
<xml_diff>
--- a/proposal_output/proposals.xlsx
+++ b/proposal_output/proposals.xlsx
@@ -578,12 +578,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Tender notice includes a specific open category (OUK/026/OP/2026-2028) for the provision of ICT Management Consulting, ICT Systems Audit, and Training on ICT Security Solutions.</t>
+          <t>Tender includes specific open categories for ICT system procurement, software, LAN/WAN services, and training on ICT security solutions.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Open to all eligible firms. Prequalification documents must be downloaded from the website and physically deposited by Thursday, 20th August 2026, 11:30 AM East African Time.</t>
+          <t>Open to eligible firms; includes reserved categories for AGPO groups (Youth, Women, and PWDs) with a valid AGPO certificate.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -609,19 +609,19 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>166f9b27c5e956f4</t>
+          <t>9cca09bd6a8caab0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Blue Dot Network Certification</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Certification</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Certification</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>https://www.bluedot-network.org/certification</t>
@@ -639,7 +639,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>apply for certification</t>
+          <t>apply for certification, certification application, certification offer</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -649,12 +649,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Matched configured ICT keyword(s): apply for certification.</t>
+          <t>Offers a certification framework and application process for infrastructure projects, which explicitly includes the ICT sector.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Review source document for eligibility requirements.</t>
+          <t>Open to infrastructure projects across major sectors, including ICT, at various lifecycle stages and ownership models.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>machine learning, artificial intelligence, grant application, funding opportunity, climate technology Africa funding</t>
+          <t>machine learning, artificial intelligence, climate technology Africa funding, grant application</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -791,12 +791,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Provides grant opportunities at the intersection of climate change and machine learning/AI, which aligns with climate technology funding keywords.</t>
+          <t>Active grant program supporting research and deployment at the intersection of climate change and machine learning.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Supports research, deployment, and dataset creation. Eligibility varies per specific call (some past calls were Africa-focused).</t>
+          <t>Supports impactful projects involving dataset creation, deployment, and research utilizing ML to tackle climate change.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Digital Health &amp; Climate Tech</t>
+          <t>Grant</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>artificial intelligence, machine learning, grant application, funding opportunity</t>
+          <t>grant application, funding opportunity, machine learning, artificial intelligence</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -862,17 +862,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Provides seed funding of up to $150K for projects leveraging artificial intelligence and machine learning to tackle climate change mitigation and adaptation.</t>
+          <t>A seed grant program supporting research, tools, and datasets at the intersection of climate change and machine learning or artificial intelligence.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Aims to build partnerships between academic researchers, non-profits, startups, and other companies. Currently has no active/future calls planned.</t>
+          <t>Currently has no active or planned future calls, though past cycles funded projects up to $150K.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Ignore</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -2791,12 +2791,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>166f9b27c5e956f4</t>
+          <t>9cca09bd6a8caab0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Certification</t>
+          <t>Blue Dot Network Certification</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">

</xml_diff>

<commit_message>
Skip JavaScript-rendered pages and merge duplicate bluedot-network.org source
Public Procurement Regulatory Authority's "Standard Tender Documents" page
renders its real content client-side (h1 is literally "Loading..."); scraping
it produced titles built from page chrome instead of real content, e.g.
"Standard Tender Documents ... Close Close ... loading... File Properties
Name File Uploader Folder". collect()/collect_raw() now detect a
JS-placeholder heading and skip the candidate entirely, since neither its
title nor its content is real. Also purged the one stale copy of this record
that had already lodged in proposal_output/proposals.json (due_date "Not
stated" meant it would never expire on its own).

Also merges the two duplicate "bluedot-network.org" source entries in
Migrations/proposal_source.json into one (both start_urls kept), which were
causing the same site to be crawled twice every run.
</commit_message>
<xml_diff>
--- a/proposal_output/proposals.xlsx
+++ b/proposal_output/proposals.xlsx
@@ -16,12 +16,12 @@
     <sheet name="Workflows" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proposals'!$A$1:$O$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proposals'!$A$1:$O$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Workplan'!$A$1:$G$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Website Register'!$A$1:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Website Register'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Keywords'!$A$1:$D$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Content Calendar'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Workflow Queue'!$A$1:$G$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Workflow Queue'!$A$1:$G$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Workflows'!$A$1:$E$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -440,12 +440,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="43" customWidth="1" min="6" max="6"/>
@@ -540,12 +540,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8d40238686713191</t>
+          <t>bc97777e6c0833cb</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Open University of Kenya Supplier Prequalification (2026-2028)</t>
+          <t>Open University of Kenya Tender Notice.pdf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -568,27 +568,27 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>training, ICT training</t>
+          <t>training</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Tender includes specific open categories for ICT system procurement, software, LAN/WAN services, and training on ICT security solutions.</t>
+          <t>Matched configured ICT keyword(s): training.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Open to eligible firms; includes reserved categories for AGPO groups (Youth, Women, and PWDs) with a valid AGPO certificate.</t>
+          <t>Review source document for eligibility requirements.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Pursue</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Digital Health &amp; Climate Tech</t>
+          <t>Data science</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -781,22 +781,22 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>machine learning, artificial intelligence, climate technology Africa funding, grant application</t>
+          <t>machine learning</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Active grant program supporting research and deployment at the intersection of climate change and machine learning.</t>
+          <t>Matched configured ICT keyword(s): machine learning.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Supports impactful projects involving dataset creation, deployment, and research utilizing ML to tackle climate change.</t>
+          <t>Review source document for eligibility requirements.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Data science</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -852,27 +852,27 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>grant application, funding opportunity, machine learning, artificial intelligence</t>
+          <t>analysis, machine learning, artificial intelligence, training</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>A seed grant program supporting research, tools, and datasets at the intersection of climate change and machine learning or artificial intelligence.</t>
+          <t>Matched configured ICT keyword(s): analysis, machine learning, artificial intelligence, training.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Currently has no active or planned future calls, though past cycles funded projects up to $150K.</t>
+          <t>Review source document for eligibility requirements.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Ignore</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1032,79 +1032,8 @@
       </c>
       <c r="O8" t="inlineStr"/>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>9b0fded721a6ff45</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Standard Tender Documents – Public Procurement Regulatory Authority × Close Close × Close Close × Close loading... File Properties Name File Uploader Folder PPA</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Training</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>https://ppra.go.ke/standard-tender-documents</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Public Procurement Regulatory Authority</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>training</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Matched configured ICT keyword(s): training.</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Review source document for eligibility requirements.</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Review required</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Project team</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="n">
-        <v>46253</v>
-      </c>
-      <c r="O9" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O9"/>
+  <autoFilter ref="A1:O8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1403,7 +1332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -1609,7 +1538,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.bluedot-network.org/certification</t>
+          <t>https://www.bluedot-network.org/certification, https://www.bluedot-network.org/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1662,31 +1591,31 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>bluedot-network.org</t>
+          <t>User submitted</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.bluedot-network.org/</t>
+          <t>https://example.gov/tenders</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>managed_source</t>
+          <t>Pending review</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Every monitor run</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Submitted 2026-08-10T09:15:56.399Z</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1696,7 +1625,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://example.gov/tenders</t>
+          <t>https://example.org/funding</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1725,7 +1654,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://example.org/funding</t>
+          <t>https://www.climatechange.ai/papers/neurips2024/98</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1742,7 +1671,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Submitted 2026-08-10T09:15:56.399Z</t>
+          <t>Submitted 2026-08-10T10:04:59.643Z</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1683,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://www.climatechange.ai/papers/neurips2024/98</t>
+          <t>https://www.climatechange.ai/papers/neurips2024/98https://www.climatechange.ai/papers/neurips2024/98</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1771,7 +1700,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Submitted 2026-08-10T10:04:59.643Z</t>
+          <t>Submitted 2026-08-10T10:11:01.745Z</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1712,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://www.climatechange.ai/papers/neurips2024/98https://www.climatechange.ai/papers/neurips2024/98</t>
+          <t>https://www.bluedot-network.org/certification</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1800,7 +1729,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Submitted 2026-08-10T10:11:01.745Z</t>
+          <t>Submitted 2026-08-11T16:20:04.680Z</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1741,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://www.bluedot-network.org/certification</t>
+          <t>https://www.climatechange.ai/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1829,7 +1758,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Submitted 2026-08-11T16:20:04.680Z</t>
+          <t>Submitted 2026-08-11T18:24:37.612Z</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1770,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://www.climatechange.ai/</t>
+          <t>https://le.ac.uk/study/international-students/countries/africa/kenya?utm_source=google-search&amp;utm_medium=paid&amp;utm_campaign=international-recruitment-2026&amp;utm_content=brand_ug-pg-ke&amp;gad_source=1&amp;gad_campaignid=22138204529&amp;gbraid=0AAAAA-Jv9mK-HMbYwd0xUiIwJsYXujvIu&amp;gclid=CjwKCAjw4dDTBhAqEiwAkHYmSix5GlL4etFz30Inndq4q0FUkb21c040s1XsfJ6nm0XAcefOUWDscRoCxsgQAvD_BwE</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1858,41 +1787,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Submitted 2026-08-11T18:24:37.612Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>User submitted</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>https://le.ac.uk/study/international-students/countries/africa/kenya?utm_source=google-search&amp;utm_medium=paid&amp;utm_campaign=international-recruitment-2026&amp;utm_content=brand_ug-pg-ke&amp;gad_source=1&amp;gad_campaignid=22138204529&amp;gbraid=0AAAAA-Jv9mK-HMbYwd0xUiIwJsYXujvIu&amp;gclid=CjwKCAjw4dDTBhAqEiwAkHYmSix5GlL4etFz30Inndq4q0FUkb21c040s1XsfJ6nm0XAcefOUWDscRoCxsgQAvD_BwE</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Pending review</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
           <t>Submitted 2026-08-11T19:52:46.857Z</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G16"/>
+  <autoFilter ref="A1:G15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2529,7 +2429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2581,12 +2481,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8d40238686713191</t>
+          <t>bc97777e6c0833cb</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Open University of Kenya Supplier Prequalification (2026-2028)</t>
+          <t>Open University of Kenya Tender Notice.pdf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2600,7 +2500,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>46253</v>
+        <v>46251</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2651,12 +2551,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>9b0fded721a6ff45</t>
+          <t>f7683a8e4ad35977</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Standard Tender Documents – Public Procurement Regulatory Authority × Close Close × Close Close × Close loading... File Properties Name File Uploader Folder PPA</t>
+          <t>Climate Change AI Grant Calls</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2679,19 +2579,19 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://ppra.go.ke/standard-tender-documents</t>
+          <t>https://www.climatechange.ai/calls</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>f7683a8e4ad35977</t>
+          <t>17124d19bfc6b3cd</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Climate Change AI Grant Calls</t>
+          <t>Climate Change AI Innovation Grants</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2714,19 +2614,19 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.climatechange.ai/calls</t>
+          <t>https://www.climatechange.ai/innovation_grants</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>17124d19bfc6b3cd</t>
+          <t>aa16da3072f3ff5b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Climate Change AI Innovation Grants</t>
+          <t>Climate Change AI Announces Innovation Grantees (April 29, 2026) | Climate Change AI</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2749,19 +2649,19 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.climatechange.ai/innovation_grants</t>
+          <t>https://www.climatechange.ai/press_releases/2026-04-29/release</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>aa16da3072f3ff5b</t>
+          <t>9cca09bd6a8caab0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Climate Change AI Announces Innovation Grantees (April 29, 2026) | Climate Change AI</t>
+          <t>Blue Dot Network Certification</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2775,7 +2675,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -2784,19 +2684,19 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.climatechange.ai/press_releases/2026-04-29/release</t>
+          <t>https://www.bluedot-network.org/certification</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>9cca09bd6a8caab0</t>
+          <t>3c2462dbed3db6a6</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Blue Dot Network Certification</t>
+          <t>OECD InfraDays 2026 Highlights the Growing Global Momentum Behind Blue Dot Network Certification</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2819,47 +2719,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.bluedot-network.org/certification</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>3c2462dbed3db6a6</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>OECD InfraDays 2026 Highlights the Growing Global Momentum Behind Blue Dot Network Certification</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Review proposal and assign a bid decision</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Project team</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>46248</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Review required</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
           <t>https://www.bluedot-network.org/news/bdn-certificationceremony</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G9"/>
+  <autoFilter ref="A1:G8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix Website Register sheet reading stale pending-source data
PENDING_SOURCE_FILE pointed at Migrations/pending_source_intake.json, the
seed template copied to the Render disk once on first boot and never
updated again, instead of proposal_output/pending_source_intake.json, the
live file the website actually reads and writes
(src/lib/source-handlers.js). The Website Register sheet's "pending review"
rows have never reflected real user submissions.

Also fixed a second bug in the same function: it listed every entry in that
file as "Pending review" regardless of its actual status, so already-
approved or already-rejected submissions showed up mislabeled as pending.
Now filters to status == "pending_review".

Verified by adding a submission to only the live file (not the template)
and confirming it now appears, then reverting the test data and generating
a real workbook to confirm the Website Register sheet is correct.
</commit_message>
<xml_diff>
--- a/proposal_output/proposals.xlsx
+++ b/proposal_output/proposals.xlsx
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proposals'!$A$1:$O$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Workplan'!$A$1:$G$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Website Register'!$A$1:$G$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Website Register'!$A$1:$G$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Keywords'!$A$1:$D$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Content Calendar'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Workflow Queue'!$A$1:$G$8</definedName>
@@ -445,7 +445,7 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="43" customWidth="1" min="6" max="6"/>
@@ -540,12 +540,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7b06c862b59f701e</t>
+          <t>bc97777e6c0833cb</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Open University of Kenya Tender Notice</t>
+          <t>Open University of Kenya Tender Notice.pdf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -573,22 +573,22 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Includes tenders for Enterprise Business Systems (ERP), Consultancy on E-Learning, and crucially Category OUK/026/OP/2026-2028: 'Training on ICT Security Solutions'.</t>
+          <t>Matched configured ICT keyword(s): training.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Open to all interested and eligible firms, with specific reservation categories for AGPO groups (Youth, Women, and PWDs) with valid certification.</t>
+          <t>Review source document for eligibility requirements.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Pursue</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -680,22 +680,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>f7683a8e4ad35977</t>
+          <t>aa16da3072f3ff5b</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Climate Change AI Grant Calls</t>
+          <t>Climate Change AI Announces Innovation Grantees (April 29, 2026) | Climate Change AI</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Digital Health &amp; Climate Tech</t>
+          <t>Data science</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.climatechange.ai/calls</t>
+          <t>https://www.climatechange.ai/press_releases/2026-04-29/release</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>machine learning, artificial intelligence, funding opportunity, grant application</t>
+          <t>analysis, machine learning, training</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -720,12 +720,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>The page lists current and past grant programs specifically focused on supporting research, deployment, and dataset creation at the intersection of climate change and machine learning/AI.</t>
+          <t>Matched configured ICT keyword(s): analysis, machine learning, training.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Supports impactful work using AI and ML for climate change solutions, though specific current call details require contacting the provider or monitoring for open rounds.</t>
+          <t>Review source document for eligibility requirements.</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -751,22 +751,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>60c52eb38ad60cf3</t>
+          <t>f7683a8e4ad35977</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Climate Change AI Innovation Grantees Announcement</t>
+          <t>Climate Change AI Grant Calls</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Digital Health &amp; Climate Tech</t>
+          <t>Data science</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.climatechange.ai/press_releases/2026-04-29/release</t>
+          <t>https://www.climatechange.ai/calls</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>machine learning, artificial intelligence, funding opportunity, grant application</t>
+          <t>machine learning</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -791,12 +791,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Provides details and profiles on active/past funding opportunities under the Climate Change AI Innovation Grants program, which focuses on machine learning solutions.</t>
+          <t>Matched configured ICT keyword(s): machine learning.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Historically supports cross-sectoral teams developing AI tools and open datasets. Call is currently closed but profiles past successful criteria.</t>
+          <t>Review source document for eligibility requirements.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Digital Health &amp; Climate Tech</t>
+          <t>Data science</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>machine learning, artificial intelligence, grant application, funding opportunity</t>
+          <t>analysis, machine learning, artificial intelligence, training</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -862,12 +862,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>A genuine funding opportunity supporting research and deployment projects that leverage artificial intelligence and machine learning to tackle climate change.</t>
+          <t>Matched configured ICT keyword(s): analysis, machine learning, artificial intelligence, training.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Supports cross-sectoral teams including academic researchers, non-profits, startups, and governmental organizations. Currently no future calls are planned, but open to partnerships.</t>
+          <t>Review source document for eligibility requirements.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1332,7 +1332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -1588,211 +1588,8 @@
       </c>
       <c r="G8" t="inlineStr"/>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>User submitted</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://example.gov/tenders</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Pending review</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Submitted 2026-08-10T09:15:56.399Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>User submitted</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://example.org/funding</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Pending review</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Submitted 2026-08-10T09:15:56.399Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>User submitted</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>https://www.climatechange.ai/papers/neurips2024/98</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Pending review</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Submitted 2026-08-10T10:04:59.643Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>User submitted</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>https://www.climatechange.ai/papers/neurips2024/98https://www.climatechange.ai/papers/neurips2024/98</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Pending review</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Submitted 2026-08-10T10:11:01.745Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>User submitted</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>https://www.bluedot-network.org/certification</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Pending review</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Submitted 2026-08-11T16:20:04.680Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>User submitted</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>https://www.climatechange.ai/</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Pending review</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Submitted 2026-08-11T18:24:37.612Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>User submitted</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>https://le.ac.uk/study/international-students/countries/africa/kenya?utm_source=google-search&amp;utm_medium=paid&amp;utm_campaign=international-recruitment-2026&amp;utm_content=brand_ug-pg-ke&amp;gad_source=1&amp;gad_campaignid=22138204529&amp;gbraid=0AAAAA-Jv9mK-HMbYwd0xUiIwJsYXujvIu&amp;gclid=CjwKCAjw4dDTBhAqEiwAkHYmSix5GlL4etFz30Inndq4q0FUkb21c040s1XsfJ6nm0XAcefOUWDscRoCxsgQAvD_BwE</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Pending review</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Submitted 2026-08-11T19:52:46.857Z</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G15"/>
+  <autoFilter ref="A1:G8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2481,12 +2278,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7b06c862b59f701e</t>
+          <t>bc97777e6c0833cb</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Open University of Kenya Tender Notice</t>
+          <t>Open University of Kenya Tender Notice.pdf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2621,12 +2418,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>60c52eb38ad60cf3</t>
+          <t>aa16da3072f3ff5b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Climate Change AI Innovation Grantees Announcement</t>
+          <t>Climate Change AI Announces Innovation Grantees (April 29, 2026) | Climate Change AI</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2640,7 +2437,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>46255</v>
+        <v>46247</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>

</xml_diff>